<commit_message>
docs(excel): agregar hipervínculos internos entre Hoja 2 y Hoja 1, y enlaces a componentes React en honeymetrics-frontend
</commit_message>
<xml_diff>
--- a/HoneyMetrics_Backlog_Scrum.xlsx
+++ b/HoneyMetrics_Backlog_Scrum.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,20 @@
       <name val="Calibri"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="5">
@@ -108,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,6 +145,18 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3536,14 +3562,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -3604,7 +3630,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Mockup / UI</t>
+          <t>Mockup / UI (React)</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -3619,7 +3645,7 @@
           <t>PB-HM-02.1</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>PB-HM-02</t>
         </is>
@@ -3650,9 +3676,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_login_3d.jpg</t>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/Login.jsx</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -3667,7 +3693,7 @@
           <t>PB-HM-07.1</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>PB-HM-07</t>
         </is>
@@ -3698,9 +3724,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_login_otp.jpg</t>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/Login.jsx</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
@@ -3715,7 +3741,7 @@
           <t>PB-HM-08.1</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>PB-HM-08</t>
         </is>
@@ -3746,9 +3772,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_qr_setup.jpg</t>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/Login.jsx</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -3763,7 +3789,7 @@
           <t>PB-HM-71.1</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>PB-HM-71</t>
         </is>
@@ -3794,9 +3820,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_threat_list.jpg</t>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/ThreatCenter.jsx</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -3811,7 +3837,7 @@
           <t>PB-HM-72.1</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>PB-HM-72</t>
         </is>
@@ -3842,9 +3868,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_threat_create.jpg</t>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>src/components/threats/ThreatModal.jsx</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
@@ -3859,7 +3885,7 @@
           <t>PB-HM-73.1</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>PB-HM-73</t>
         </is>
@@ -3890,9 +3916,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_threat_edit.jpg</t>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>src/components/threats/ThreatModal.jsx</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
@@ -3907,7 +3933,7 @@
           <t>PB-HM-74.1</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>PB-HM-74</t>
         </is>
@@ -3938,9 +3964,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_threat_delete.jpg</t>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/ThreatCenter.jsx</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
@@ -3955,7 +3981,7 @@
           <t>PB-HM-62.1</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>PB-HM-62</t>
         </is>
@@ -3986,9 +4012,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_botnet_alert.jpg</t>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>src/components/threats/BotnetAlertBadge.jsx</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
@@ -4003,7 +4029,7 @@
           <t>PB-HM-63.1</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>PB-HM-63</t>
         </is>
@@ -4034,9 +4060,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_bot_classifier.jpg</t>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>src/components/threats/ThreatScoreCard.jsx</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -4051,7 +4077,7 @@
           <t>PB-HM-26.1</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>PB-HM-26</t>
         </is>
@@ -4082,9 +4108,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_plotly_dashboard.jpg</t>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/DashboardPage.jsx</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
@@ -4099,7 +4125,7 @@
           <t>PB-HM-27.1</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>PB-HM-27</t>
         </is>
@@ -4130,9 +4156,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_time_filter.jpg</t>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>src/components/dashboard/PlotlyCharts.jsx</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
@@ -4147,7 +4173,7 @@
           <t>PB-HM-70.1</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>PB-HM-70</t>
         </is>
@@ -4178,9 +4204,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_predictive_heatmap.jpg</t>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>src/components/dashboard/PlotlyCharts.jsx</t>
         </is>
       </c>
       <c r="J16" s="9" t="inlineStr">
@@ -4195,7 +4221,7 @@
           <t>PB-HM-37.1</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>PB-HM-37</t>
         </is>
@@ -4226,9 +4252,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_async_export.jpg</t>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/LogsReport.jsx</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
@@ -4243,7 +4269,7 @@
           <t>PB-HM-38.1</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>PB-HM-38</t>
         </is>
@@ -4274,9 +4300,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_export_history.jpg</t>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/LogsReport.jsx</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
@@ -4291,7 +4317,7 @@
           <t>PB-HM-39.1</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>PB-HM-39</t>
         </is>
@@ -4322,9 +4348,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_jsonl_download.jpg</t>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/LogsReport.jsx</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -4339,7 +4365,7 @@
           <t>PB-HM-40.1</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>PB-HM-40</t>
         </is>
@@ -4370,9 +4396,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_telegram_approval.jpg</t>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>src/components/logs/ExportModal.jsx</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
@@ -4387,7 +4413,7 @@
           <t>PB-HM-42.1</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>PB-HM-42</t>
         </is>
@@ -4418,9 +4444,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_pdf_generator.jpg</t>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>src/utils/PdfGenerator.js</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -4435,7 +4461,7 @@
           <t>PB-HM-44.1</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>PB-HM-44</t>
         </is>
@@ -4466,9 +4492,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_spike_alert.jpg</t>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>src/components/layout/StatusBanner.jsx</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
@@ -4483,7 +4509,7 @@
           <t>PB-HM-65.1</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>PB-HM-65</t>
         </is>
@@ -4514,9 +4540,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_honeypot_advisor.jpg</t>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/DashboardMock.jsx</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -4531,7 +4557,7 @@
           <t>PB-HM-64.1</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>PB-HM-64</t>
         </is>
@@ -4562,9 +4588,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_patch_intel.jpg</t>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/Dashboard.jsx</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
@@ -4579,7 +4605,7 @@
           <t>PB-HM-66.1</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>PB-HM-66</t>
         </is>
@@ -4610,9 +4636,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_fim_timeline.jpg</t>
+      <c r="I25" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/ThreatCenter.jsx</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -4627,7 +4653,7 @@
           <t>PB-HM-67.1</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>PB-HM-67</t>
         </is>
@@ -4658,9 +4684,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>N/A (Lógica backend)</t>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>src/mocks/threatsDatabase.js</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr">
@@ -4675,7 +4701,7 @@
           <t>PB-HM-67.2</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>PB-HM-67</t>
         </is>
@@ -4706,9 +4732,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_kill_chain_ui.jpg</t>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/ThreatCenter.jsx</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -4723,7 +4749,7 @@
           <t>PB-HM-68.1</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>PB-HM-68</t>
         </is>
@@ -4754,9 +4780,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_hitl_rootcheck.jpg</t>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/ThreatCenter.jsx</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr">
@@ -4771,7 +4797,7 @@
           <t>PB-HM-69.1</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>PB-HM-69</t>
         </is>
@@ -4802,9 +4828,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>mockups/mockup_cis_compliance.jpg</t>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>src/pages/DashboardMock.jsx</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
@@ -4819,7 +4845,7 @@
           <t>PB-HM-48.1</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>PB-HM-48</t>
         </is>
@@ -4850,9 +4876,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I30" s="8" t="inlineStr">
-        <is>
-          <t>mockups/mockup_ml_metrics.jpg</t>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>src/pages/DashboardMock.jsx</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr">
@@ -4867,7 +4893,7 @@
           <t>PB-HM-56.1</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>PB-HM-56</t>
         </is>
@@ -4898,9 +4924,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>N/A (Lógica global)</t>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>src/context/AuthContext.jsx</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
@@ -4910,6 +4936,62 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId54"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: actualizar PB-HM-06 con tareas de correo transaccional (Resend + Cloudflare) y contingencia M365
</commit_message>
<xml_diff>
--- a/HoneyMetrics_Backlog_Scrum.xlsx
+++ b/HoneyMetrics_Backlog_Scrum.xlsx
@@ -2758,9 +2758,9 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>- [ ] Diseñar e implementar el componente UI necesario
-- [ ] Establecer lógica de estado (React hooks) y validaciones
-- [ ] Conectar la interfaz con la API Backend correspondiente</t>
+          <t>- [ ] Configurar proveedor de correos transaccionales (Resend) y verificar dominio `johan-d3v.site` en Cloudflare (registros SPF, DKIM, DMARC).
+- [ ] Plan de Contingencia (Opción B): Si fallan los filtros universitarios, documentar e implementar envío de correos vía Microsoft Graph API usando un entorno M365 Developer.
+- [ ] Integrar SDK de correo en FastAPI y conectar UI (React) para solicitar y procesar el token de recuperación de contraseña.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">

</xml_diff>